<commit_message>
MACD scan results 2026-08-28
</commit_message>
<xml_diff>
--- a/results/macd_2026-08-28.xlsx
+++ b/results/macd_2026-08-28.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,7 +458,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ABCL</t>
+          <t>ABUS</t>
         </is>
       </c>
     </row>
@@ -466,7 +466,7 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CELC</t>
+          <t>CENX</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -477,7 +477,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ABSI</t>
+          <t>ALM</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ABUS</t>
+          <t>AQST</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>IMTX</t>
+          <t>META</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -515,7 +515,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>ARGX</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>AQST</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
@@ -549,7 +549,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ARGX</t>
+          <t>CADL</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>AU</t>
+          <t>CARG</t>
         </is>
       </c>
     </row>
@@ -579,7 +579,7 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>AVAH</t>
+          <t>CCEP</t>
         </is>
       </c>
     </row>
@@ -588,13 +588,13 @@
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>CACC</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>CGAU</t>
         </is>
       </c>
     </row>
@@ -603,13 +603,13 @@
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CNR</t>
+          <t>CDNA</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CACC</t>
+          <t>CRWD</t>
         </is>
       </c>
     </row>
@@ -618,13 +618,13 @@
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>CHRD</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CADL</t>
+          <t>ERAS</t>
         </is>
       </c>
     </row>
@@ -633,13 +633,13 @@
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>CNR</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CGAU</t>
+          <t>EXEL</t>
         </is>
       </c>
     </row>
@@ -648,13 +648,13 @@
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
-          <t>DJCO</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CLPT</t>
+          <t>EZPW</t>
         </is>
       </c>
     </row>
@@ -663,13 +663,13 @@
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ERAS</t>
+          <t>CVSA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CMPS</t>
+          <t>FA</t>
         </is>
       </c>
     </row>
@@ -678,13 +678,13 @@
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>DASH</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>FCFS</t>
         </is>
       </c>
     </row>
@@ -693,13 +693,13 @@
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
-          <t>EZPW</t>
+          <t>DJCO</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>GRAL</t>
         </is>
       </c>
     </row>
@@ -708,13 +708,13 @@
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>FRHC</t>
+          <t>ETSY</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>HOOD</t>
         </is>
       </c>
     </row>
@@ -729,7 +729,7 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>IBKR</t>
         </is>
       </c>
     </row>
@@ -744,7 +744,7 @@
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>FCFS</t>
+          <t>IBRX</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>GH</t>
+          <t>IDYA</t>
         </is>
       </c>
     </row>
@@ -768,13 +768,13 @@
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>KRNY</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>IFRX</t>
         </is>
       </c>
     </row>
@@ -783,13 +783,13 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>IBKR</t>
+          <t>LECO</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>ILMN</t>
         </is>
       </c>
     </row>
@@ -798,13 +798,13 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>IBRX</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>INBX</t>
         </is>
       </c>
     </row>
@@ -813,13 +813,13 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>MDGL</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>HSIC</t>
+          <t>JOYY</t>
         </is>
       </c>
     </row>
@@ -828,13 +828,13 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>INBX</t>
+          <t>NEO</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>IDYA</t>
+          <t>KRYS</t>
         </is>
       </c>
     </row>
@@ -843,13 +843,13 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>IRON</t>
+          <t>NTNX</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>IFRX</t>
+          <t>MELI</t>
         </is>
       </c>
     </row>
@@ -858,13 +858,13 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>KRNY</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>IMMX</t>
+          <t>NDAQ</t>
         </is>
       </c>
     </row>
@@ -873,13 +873,13 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>KRYS</t>
+          <t>NWSA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>JOYY</t>
+          <t>NEXT</t>
         </is>
       </c>
     </row>
@@ -888,13 +888,13 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>LECO</t>
+          <t>OKTA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>LPTH</t>
+          <t>PLTR</t>
         </is>
       </c>
     </row>
@@ -903,13 +903,13 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>PAA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>LTRX</t>
+          <t>PTEN</t>
         </is>
       </c>
     </row>
@@ -918,13 +918,13 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MDGL</t>
+          <t>PAGP</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>PVLA</t>
         </is>
       </c>
     </row>
@@ -933,13 +933,13 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>SBRA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>REAX</t>
         </is>
       </c>
     </row>
@@ -948,13 +948,13 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>NEO</t>
+          <t>SBUX</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>NTRA</t>
+          <t>RGLD</t>
         </is>
       </c>
     </row>
@@ -963,13 +963,13 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>NEXT</t>
+          <t>SLAB</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>SBLK</t>
         </is>
       </c>
     </row>
@@ -978,13 +978,13 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>NWS</t>
+          <t>SMTC</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>OVID</t>
+          <t>SEIC</t>
         </is>
       </c>
     </row>
@@ -993,13 +993,13 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>TH</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>SRRK</t>
         </is>
       </c>
     </row>
@@ -1008,13 +1008,13 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>OKTA</t>
+          <t>TRMD</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>PHVS</t>
+          <t>SSRM</t>
         </is>
       </c>
     </row>
@@ -1023,13 +1023,13 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>VCTR</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>TEM</t>
         </is>
       </c>
     </row>
@@ -1038,196 +1038,46 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>XMTR</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>TGTX</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>ROIV</t>
-        </is>
-      </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>REAX</t>
+          <t>TPG</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>RVMD</t>
-        </is>
-      </c>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>RGLD</t>
+          <t>TRLV</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>SBUX</t>
-        </is>
-      </c>
+      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>RPRX</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr"/>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>SLAB</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>RZLT</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr"/>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>SLDB</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>SBLK</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr"/>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>SLS</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>SBRA</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr"/>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>SMTC</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>SEIC</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr"/>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>TGTX</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>SRRK</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr"/>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>TH</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>SSRM</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>TRMD</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>TEM</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr"/>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>TRLV</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr"/>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr">
-        <is>
           <t>VSXY</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr"/>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>XNCR</t>
         </is>
       </c>
     </row>

</xml_diff>